<commit_message>
Selecting all legacy questions with no Regions
</commit_message>
<xml_diff>
--- a/data/exams/chemistry/Chemistry2020LegacyMetadata.xlsx
+++ b/data/exams/chemistry/Chemistry2020LegacyMetadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Exam\data\exams\chemistry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78888AD1-B5DD-4C74-9A8B-9EDE4AE09175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF18FAA-90E5-4632-9E47-A4D4883E3D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2B4427A6-DBD2-467C-BF3E-C0AF149C4F60}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2B4427A6-DBD2-467C-BF3E-C0AF149C4F60}"/>
   </bookViews>
   <sheets>
     <sheet name="QCAA" sheetId="1" r:id="rId1"/>
@@ -613,12 +613,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ADA3352-68AE-4661-810A-6C445B58AD44}">
   <dimension ref="A1:G60"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="5" width="9" style="2"/>
+    <col min="6" max="7" width="8.796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -641,7 +642,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2020</v>
       </c>
@@ -657,11 +658,11 @@
       <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2020</v>
       </c>
@@ -677,11 +678,11 @@
       <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -697,11 +698,11 @@
       <c r="E4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -717,11 +718,11 @@
       <c r="E5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2020</v>
       </c>
@@ -737,11 +738,11 @@
       <c r="E6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2020</v>
       </c>
@@ -757,11 +758,11 @@
       <c r="E7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2020</v>
       </c>
@@ -777,11 +778,11 @@
       <c r="E8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2020</v>
       </c>
@@ -797,11 +798,11 @@
       <c r="E9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2020</v>
       </c>
@@ -817,11 +818,11 @@
       <c r="E10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2020</v>
       </c>
@@ -837,11 +838,11 @@
       <c r="E11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2020</v>
       </c>
@@ -857,11 +858,11 @@
       <c r="E12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2020</v>
       </c>
@@ -877,11 +878,11 @@
       <c r="E13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2020</v>
       </c>
@@ -897,11 +898,11 @@
       <c r="E14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2020</v>
       </c>
@@ -917,11 +918,11 @@
       <c r="E15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2020</v>
       </c>
@@ -937,11 +938,11 @@
       <c r="E16" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2020</v>
       </c>
@@ -957,11 +958,11 @@
       <c r="E17" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2020</v>
       </c>
@@ -977,11 +978,11 @@
       <c r="E18" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2020</v>
       </c>
@@ -997,11 +998,11 @@
       <c r="E19" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2020</v>
       </c>
@@ -1017,11 +1018,11 @@
       <c r="E20" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2020</v>
       </c>
@@ -1037,11 +1038,11 @@
       <c r="E21" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2020</v>
       </c>
@@ -1058,7 +1059,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2020</v>
       </c>
@@ -1075,7 +1076,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2020</v>
       </c>
@@ -1091,11 +1092,11 @@
       <c r="E24" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G24" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2020</v>
       </c>
@@ -1111,11 +1112,11 @@
       <c r="E25" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G25" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2020</v>
       </c>
@@ -1131,11 +1132,11 @@
       <c r="E26" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G26" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2020</v>
       </c>
@@ -1152,7 +1153,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2020</v>
       </c>
@@ -1169,7 +1170,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>2020</v>
       </c>
@@ -1185,11 +1186,11 @@
       <c r="E29" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G29" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>2020</v>
       </c>
@@ -1205,11 +1206,11 @@
       <c r="E30" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G30" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>2020</v>
       </c>
@@ -1225,11 +1226,11 @@
       <c r="E31" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G31" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>2020</v>
       </c>
@@ -1245,11 +1246,11 @@
       <c r="E32" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G32" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>2020</v>
       </c>
@@ -1265,11 +1266,11 @@
       <c r="E33" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G33" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>2020</v>
       </c>
@@ -1289,7 +1290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>2020</v>
       </c>
@@ -1305,11 +1306,11 @@
       <c r="E35" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G35" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>2020</v>
       </c>
@@ -1325,11 +1326,11 @@
       <c r="E36" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G36" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>2020</v>
       </c>
@@ -1345,11 +1346,11 @@
       <c r="E37" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G37" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>2020</v>
       </c>
@@ -1365,11 +1366,11 @@
       <c r="E38" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G38" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>2020</v>
       </c>
@@ -1385,11 +1386,11 @@
       <c r="E39" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G39" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>2020</v>
       </c>
@@ -1405,11 +1406,11 @@
       <c r="E40" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G40" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>2020</v>
       </c>
@@ -1425,11 +1426,11 @@
       <c r="E41" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G41">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G41" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>2020</v>
       </c>
@@ -1445,11 +1446,11 @@
       <c r="E42" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G42">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G42" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>2020</v>
       </c>
@@ -1465,11 +1466,11 @@
       <c r="E43" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G43">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G43" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>2020</v>
       </c>
@@ -1485,11 +1486,11 @@
       <c r="E44" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G44" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>2020</v>
       </c>
@@ -1505,11 +1506,11 @@
       <c r="E45" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G45">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G45" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>2020</v>
       </c>
@@ -1525,11 +1526,11 @@
       <c r="E46" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G46">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G46" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>2020</v>
       </c>
@@ -1545,11 +1546,11 @@
       <c r="E47" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G47" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>2020</v>
       </c>
@@ -1565,11 +1566,11 @@
       <c r="E48" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G48">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G48" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>2020</v>
       </c>
@@ -1585,11 +1586,11 @@
       <c r="E49" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G49" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>2020</v>
       </c>
@@ -1605,11 +1606,11 @@
       <c r="E50" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G50">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G50" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>2020</v>
       </c>
@@ -1625,11 +1626,11 @@
       <c r="E51" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G51">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G51" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>2020</v>
       </c>
@@ -1645,11 +1646,11 @@
       <c r="E52" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G52">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G52" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>2020</v>
       </c>
@@ -1665,11 +1666,11 @@
       <c r="E53" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G53">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G53" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>2020</v>
       </c>
@@ -1685,11 +1686,11 @@
       <c r="E54" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G54">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G54" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>2020</v>
       </c>
@@ -1705,11 +1706,11 @@
       <c r="E55" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G55">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G55" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>2020</v>
       </c>
@@ -1725,11 +1726,11 @@
       <c r="E56" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G56">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G56" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>2020</v>
       </c>
@@ -1745,11 +1746,11 @@
       <c r="E57" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G57">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G57" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>2020</v>
       </c>
@@ -1765,11 +1766,11 @@
       <c r="E58" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G58">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G58" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>2020</v>
       </c>
@@ -1785,11 +1786,11 @@
       <c r="E59" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G59">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G59" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>2020</v>
       </c>
@@ -1805,7 +1806,7 @@
       <c r="E60" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G60">
+      <c r="G60" s="2">
         <v>1</v>
       </c>
     </row>

</xml_diff>